<commit_message>
Clean up project structure
</commit_message>
<xml_diff>
--- a/CoursePatterns/Output/subject_taken_together.xlsx
+++ b/CoursePatterns/Output/subject_taken_together.xlsx
@@ -1849,7 +1849,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>COSE214, COSE222, COSE371</t>
+          <t>COSE342, COSE371</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1858,7 +1858,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.6279</v>
+        <v>0.6512</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -1870,7 +1870,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>COSE214, COSE215</t>
+          <t>COSE214, COSE342, COSE371</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1879,7 +1879,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.6744</v>
+        <v>0.6279</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -1891,7 +1891,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>COSE215, COSE222</t>
+          <t>COSE214, COSE215</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1900,7 +1900,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.6047</v>
+        <v>0.6744</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -1912,7 +1912,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>COSE371</t>
+          <t>COSE211, COSE371</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.6977</v>
+        <v>0.6047</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
@@ -1933,7 +1933,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>COSE222, COSE342, COSE371</t>
+          <t>COSE341, COSE342, COSE371</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1954,7 +1954,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>COSE214, COSE341, COSE371</t>
+          <t>COSE371</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1963,7 +1963,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.6279</v>
+        <v>0.6977</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -1975,7 +1975,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>COSE214, COSE371</t>
+          <t>COSE211, COSE214, COSE215</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1984,7 +1984,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.6744</v>
+        <v>0.6512</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
@@ -1996,7 +1996,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>COSE342, COSE371</t>
+          <t>COSE222, COSE341, COSE371</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2005,7 +2005,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.6512</v>
+        <v>0.6047</v>
       </c>
       <c r="D9" t="n">
         <v>1</v>
@@ -2017,7 +2017,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>COSE214, COSE342, COSE371</t>
+          <t>COSE222, COSE342, COSE371</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2026,7 +2026,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.6279</v>
+        <v>0.6047</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
@@ -2059,7 +2059,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>COSE222, COSE341, COSE371</t>
+          <t>COSE341, COSE371</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2068,7 +2068,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.6047</v>
+        <v>0.6512</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -2080,7 +2080,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>COSE341, COSE342, COSE371</t>
+          <t>COSE215, COSE222</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2101,7 +2101,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>COSE211, COSE371</t>
+          <t>COSE214, COSE222, COSE371</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2110,7 +2110,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.6047</v>
+        <v>0.6279</v>
       </c>
       <c r="D14" t="n">
         <v>1</v>
@@ -2122,7 +2122,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>COSE341, COSE371</t>
+          <t>COSE214, COSE341, COSE371</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2131,7 +2131,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.6512</v>
+        <v>0.6279</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -2143,7 +2143,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>COSE211, COSE214, COSE215</t>
+          <t>COSE214, COSE371</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2152,7 +2152,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.6512</v>
+        <v>0.6744</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
@@ -2227,12 +2227,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>COSE211, COSE213</t>
+          <t>COSE211, COSE214</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2242,18 +2242,18 @@
         <v>0.9714</v>
       </c>
       <c r="E20" t="n">
-        <v>1.0711</v>
+        <v>1.0443</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>COSE214, COSE222</t>
+          <t>COSE211, COSE213</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2263,13 +2263,13 @@
         <v>0.9714</v>
       </c>
       <c r="E21" t="n">
-        <v>1.0443</v>
+        <v>1.0711</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>COSE211, COSE214</t>
+          <t>COSE214, COSE222</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2416,12 +2416,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>COSE211, COSE341</t>
+          <t>COSE214, COSE222, COSE341</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -2431,18 +2431,18 @@
         <v>0.9687</v>
       </c>
       <c r="E29" t="n">
-        <v>1.0681</v>
+        <v>1.0414</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>COSE341, COSE342</t>
+          <t>COSE213, COSE222, COSE341</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -2452,13 +2452,13 @@
         <v>0.9687</v>
       </c>
       <c r="E30" t="n">
-        <v>1.0414</v>
+        <v>1.0681</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>COSE222, COSE342</t>
+          <t>COSE341, COSE342</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2479,7 +2479,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>COSE341, COSE342</t>
+          <t>COSE211, COSE341</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2500,7 +2500,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>COSE214, COSE222, COSE341</t>
+          <t>COSE341, COSE342</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2521,7 +2521,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>COSE213, COSE222, COSE341</t>
+          <t>COSE211, COSE222</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2542,12 +2542,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>COSE211, COSE222</t>
+          <t>COSE222, COSE342</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -2557,7 +2557,7 @@
         <v>0.9687</v>
       </c>
       <c r="E35" t="n">
-        <v>1.0414</v>
+        <v>1.0681</v>
       </c>
     </row>
     <row r="36">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -2620,18 +2620,18 @@
         <v>0.9687</v>
       </c>
       <c r="E38" t="n">
-        <v>1.0681</v>
+        <v>1.0414</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE222</t>
+          <t>COSE214, COSE221</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -2641,13 +2641,13 @@
         <v>0.9677</v>
       </c>
       <c r="E39" t="n">
-        <v>1.067</v>
+        <v>1.1559</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE341</t>
+          <t>COSE221, COSE222</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2710,12 +2710,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>COSE221, COSE222</t>
+          <t>COSE211, COSE213, COSE222</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -2725,13 +2725,13 @@
         <v>0.9677</v>
       </c>
       <c r="E43" t="n">
-        <v>1.0403</v>
+        <v>1.067</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>COSE214, COSE221</t>
+          <t>COSE221, COSE222</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2752,7 +2752,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>COSE221, COSE222</t>
+          <t>COSE211, COSE213, COSE341</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2773,12 +2773,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>COSE213, COSE222, COSE342</t>
+          <t>COSE214, COSE222, COSE342</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -2788,13 +2788,13 @@
         <v>0.9677</v>
       </c>
       <c r="E46" t="n">
-        <v>1.067</v>
+        <v>1.0403</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>COSE214, COSE222, COSE342</t>
+          <t>COSE214, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2815,7 +2815,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>COSE214, COSE221</t>
+          <t>COSE213, COSE221</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2857,12 +2857,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>COSE213, COSE221</t>
+          <t>COSE213, COSE222, COSE342</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -2872,18 +2872,18 @@
         <v>0.9677</v>
       </c>
       <c r="E50" t="n">
-        <v>1.1559</v>
+        <v>1.067</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>COSE213, COSE341, COSE342</t>
+          <t>COSE214, COSE221</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -2893,7 +2893,7 @@
         <v>0.9677</v>
       </c>
       <c r="E51" t="n">
-        <v>1.067</v>
+        <v>1.0403</v>
       </c>
     </row>
     <row r="52">
@@ -2920,12 +2920,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>COSE214, COSE341, COSE342</t>
+          <t>COSE215</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE211</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -2935,18 +2935,18 @@
         <v>0.9677</v>
       </c>
       <c r="E53" t="n">
-        <v>1.0403</v>
+        <v>1.1247</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>COSE215</t>
+          <t>COSE213, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>COSE211</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -2956,13 +2956,13 @@
         <v>0.9677</v>
       </c>
       <c r="E54" t="n">
-        <v>1.1247</v>
+        <v>1.067</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE342</t>
+          <t>COSE371</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2983,12 +2983,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>COSE211, COSE214, COSE342</t>
+          <t>COSE211, COSE213, COSE342</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -2998,18 +2998,18 @@
         <v>0.9667</v>
       </c>
       <c r="E56" t="n">
-        <v>1.0392</v>
+        <v>1.0658</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>COSE371</t>
+          <t>COSE211, COSE214, COSE342</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -3019,7 +3019,7 @@
         <v>0.9667</v>
       </c>
       <c r="E57" t="n">
-        <v>1.0658</v>
+        <v>1.0392</v>
       </c>
     </row>
     <row r="58">
@@ -3046,12 +3046,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>COSE211, COSE222, COSE341</t>
+          <t>COSE211, COSE215</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -3061,18 +3061,18 @@
         <v>0.9667</v>
       </c>
       <c r="E59" t="n">
-        <v>1.0658</v>
+        <v>1.0392</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>COSE371</t>
+          <t>COSE222, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>COSE213, COSE214</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -3082,13 +3082,13 @@
         <v>0.9667</v>
       </c>
       <c r="E60" t="n">
-        <v>1.0939</v>
+        <v>1.0658</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>COSE213, COSE221, COSE222</t>
+          <t>COSE211, COSE222, COSE341</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3109,12 +3109,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>COSE214, COSE221, COSE222</t>
+          <t>COSE213, COSE215</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -3124,7 +3124,7 @@
         <v>0.9667</v>
       </c>
       <c r="E62" t="n">
-        <v>1.0392</v>
+        <v>1.0658</v>
       </c>
     </row>
     <row r="63">
@@ -3151,12 +3151,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>COSE213, COSE215</t>
+          <t>COSE214, COSE221, COSE222</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -3166,18 +3166,18 @@
         <v>0.9667</v>
       </c>
       <c r="E64" t="n">
-        <v>1.0658</v>
+        <v>1.0392</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>COSE222, COSE341, COSE342</t>
+          <t>COSE213, COSE221, COSE222</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -3187,18 +3187,18 @@
         <v>0.9667</v>
       </c>
       <c r="E65" t="n">
-        <v>1.0392</v>
+        <v>1.0658</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>COSE213, COSE215</t>
+          <t>COSE213, COSE371</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>COSE211</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -3208,18 +3208,18 @@
         <v>0.9667</v>
       </c>
       <c r="E66" t="n">
-        <v>1.1234</v>
+        <v>1.0658</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>COSE222, COSE341, COSE342</t>
+          <t>COSE213, COSE215</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE211</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -3229,18 +3229,18 @@
         <v>0.9667</v>
       </c>
       <c r="E67" t="n">
-        <v>1.0658</v>
+        <v>1.1234</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>COSE213, COSE371</t>
+          <t>COSE222, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -3250,18 +3250,18 @@
         <v>0.9667</v>
       </c>
       <c r="E68" t="n">
-        <v>1.0658</v>
+        <v>1.0392</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>COSE211, COSE215</t>
+          <t>COSE371</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE213, COSE214</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -3271,18 +3271,18 @@
         <v>0.9667</v>
       </c>
       <c r="E69" t="n">
-        <v>1.0392</v>
+        <v>1.0939</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>COSE211, COSE341, COSE342</t>
+          <t>COSE221, COSE341</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -3292,18 +3292,18 @@
         <v>0.9655</v>
       </c>
       <c r="E70" t="n">
-        <v>1.0645</v>
+        <v>1.1533</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>COSE214, COSE222, COSE341, COSE342</t>
+          <t>COSE211, COSE213, COSE215</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -3313,18 +3313,18 @@
         <v>0.9655</v>
       </c>
       <c r="E71" t="n">
-        <v>1.0379</v>
+        <v>1.0645</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>COSE221, COSE341</t>
+          <t>COSE214, COSE222, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -3334,18 +3334,18 @@
         <v>0.9655</v>
       </c>
       <c r="E72" t="n">
-        <v>1.1533</v>
+        <v>1.0379</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>COSE214, COSE215</t>
+          <t>COSE213, COSE214, COSE215</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>COSE211, COSE213</t>
+          <t>COSE211</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -3355,18 +3355,18 @@
         <v>0.9655</v>
       </c>
       <c r="E73" t="n">
-        <v>1.1862</v>
+        <v>1.1221</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>COSE211, COSE214, COSE222, COSE341</t>
+          <t>COSE214, COSE215</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE211, COSE213</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -3376,18 +3376,18 @@
         <v>0.9655</v>
       </c>
       <c r="E74" t="n">
-        <v>1.0379</v>
+        <v>1.1862</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>COSE213, COSE214, COSE215</t>
+          <t>COSE221, COSE341</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>COSE211</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -3397,7 +3397,7 @@
         <v>0.9655</v>
       </c>
       <c r="E75" t="n">
-        <v>1.1221</v>
+        <v>1.0645</v>
       </c>
     </row>
     <row r="76">
@@ -3445,7 +3445,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE215</t>
+          <t>COSE211, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3466,7 +3466,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>COSE221, COSE341</t>
+          <t>COSE211, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3487,12 +3487,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>COSE211, COSE341, COSE342</t>
+          <t>COSE211, COSE213, COSE222, COSE341</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -3502,18 +3502,18 @@
         <v>0.9655</v>
       </c>
       <c r="E80" t="n">
-        <v>1.0379</v>
+        <v>1.0645</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>COSE221, COSE341</t>
+          <t>COSE211, COSE214, COSE222, COSE341</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -3523,18 +3523,18 @@
         <v>0.9655</v>
       </c>
       <c r="E81" t="n">
-        <v>1.0645</v>
+        <v>1.0379</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE222, COSE341</t>
+          <t>COSE221, COSE341</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -3544,13 +3544,13 @@
         <v>0.9655</v>
       </c>
       <c r="E82" t="n">
-        <v>1.0645</v>
+        <v>1.0379</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>COSE213, COSE341, COSE371</t>
+          <t>COSE342, COSE371</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3571,12 +3571,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>COSE342, COSE371</t>
+          <t>COSE211, COSE214, COSE221</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>COSE213, COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -3586,18 +3586,18 @@
         <v>0.9643</v>
       </c>
       <c r="E84" t="n">
-        <v>1.0912</v>
+        <v>1.0366</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>COSE211, COSE221, COSE222</t>
+          <t>COSE213, COSE222, COSE371</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -3607,18 +3607,18 @@
         <v>0.9643</v>
       </c>
       <c r="E85" t="n">
-        <v>1.0366</v>
+        <v>1.0632</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>COSE213, COSE342, COSE371</t>
+          <t>COSE222, COSE371</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213, COSE214</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -3628,18 +3628,18 @@
         <v>0.9643</v>
       </c>
       <c r="E86" t="n">
-        <v>1.0632</v>
+        <v>1.0912</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>COSE341, COSE371</t>
+          <t>COSE213, COSE341, COSE371</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>COSE213, COSE214</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -3649,7 +3649,7 @@
         <v>0.9643</v>
       </c>
       <c r="E87" t="n">
-        <v>1.0912</v>
+        <v>1.0632</v>
       </c>
     </row>
     <row r="88">
@@ -3676,12 +3676,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE221</t>
+          <t>COSE213, COSE342, COSE371</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -3691,18 +3691,18 @@
         <v>0.9643</v>
       </c>
       <c r="E89" t="n">
-        <v>1.1518</v>
+        <v>1.0632</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>COSE222, COSE371</t>
+          <t>COSE221, COSE222, COSE341</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -3712,18 +3712,18 @@
         <v>0.9643</v>
       </c>
       <c r="E90" t="n">
-        <v>1.0632</v>
+        <v>1.0366</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>COSE213, COSE221, COSE341</t>
+          <t>COSE341, COSE371</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE213, COSE214</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -3733,18 +3733,18 @@
         <v>0.9643</v>
       </c>
       <c r="E91" t="n">
-        <v>1.1518</v>
+        <v>1.0912</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>COSE211, COSE214, COSE221</t>
+          <t>COSE211, COSE213, COSE221</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -3754,18 +3754,18 @@
         <v>0.9643</v>
       </c>
       <c r="E92" t="n">
-        <v>1.0366</v>
+        <v>1.1518</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>COSE211, COSE221, COSE222</t>
+          <t>COSE211, COSE222, COSE342</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -3775,18 +3775,18 @@
         <v>0.9643</v>
       </c>
       <c r="E93" t="n">
-        <v>1.0632</v>
+        <v>1.1207</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>COSE211, COSE214, COSE221</t>
+          <t>COSE211, COSE222, COSE342</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -3796,18 +3796,18 @@
         <v>0.9643</v>
       </c>
       <c r="E94" t="n">
-        <v>1.1518</v>
+        <v>1.0366</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>COSE211, COSE222, COSE342</t>
+          <t>COSE211, COSE214, COSE221</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -3817,18 +3817,18 @@
         <v>0.9643</v>
       </c>
       <c r="E95" t="n">
-        <v>1.0366</v>
+        <v>1.1518</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>COSE221, COSE222, COSE341</t>
+          <t>COSE211, COSE213, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -3838,18 +3838,18 @@
         <v>0.9643</v>
       </c>
       <c r="E96" t="n">
-        <v>1.0366</v>
+        <v>1.0632</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE221</t>
+          <t>COSE214, COSE221, COSE341</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -3859,13 +3859,13 @@
         <v>0.9643</v>
       </c>
       <c r="E97" t="n">
-        <v>1.0632</v>
+        <v>1.0366</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>COSE213, COSE222, COSE371</t>
+          <t>COSE213, COSE221, COSE341</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -3907,12 +3907,12 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>COSE213, COSE221, COSE341</t>
+          <t>COSE214, COSE221, COSE341</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -3922,18 +3922,18 @@
         <v>0.9643</v>
       </c>
       <c r="E100" t="n">
-        <v>1.0632</v>
+        <v>1.1518</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>COSE222, COSE371</t>
+          <t>COSE211, COSE214, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>COSE213, COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -3943,18 +3943,18 @@
         <v>0.9643</v>
       </c>
       <c r="E101" t="n">
-        <v>1.0912</v>
+        <v>1.0366</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>COSE214, COSE221, COSE341</t>
+          <t>COSE211, COSE221, COSE222</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -3964,18 +3964,18 @@
         <v>0.9643</v>
       </c>
       <c r="E102" t="n">
-        <v>1.0366</v>
+        <v>1.0632</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>COSE211, COSE222, COSE342</t>
+          <t>COSE221, COSE222, COSE341</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -3985,13 +3985,13 @@
         <v>0.9643</v>
       </c>
       <c r="E103" t="n">
-        <v>1.1207</v>
+        <v>1.0632</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>COSE214, COSE221, COSE341</t>
+          <t>COSE213, COSE221, COSE341</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -4012,7 +4012,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>COSE342, COSE371</t>
+          <t>COSE222, COSE371</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -4033,12 +4033,12 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE341, COSE342</t>
+          <t>COSE342, COSE371</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213, COSE214</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -4048,13 +4048,13 @@
         <v>0.9643</v>
       </c>
       <c r="E106" t="n">
-        <v>1.0632</v>
+        <v>1.0912</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>COSE211, COSE214, COSE341, COSE342</t>
+          <t>COSE211, COSE221, COSE222</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -4075,7 +4075,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>COSE221, COSE222, COSE341</t>
+          <t>COSE211, COSE213, COSE221</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -4096,7 +4096,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>COSE214, COSE221, COSE222, COSE341</t>
+          <t>COSE214, COSE221, COSE342</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -4117,7 +4117,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>COSE211, COSE214, COSE222, COSE342</t>
+          <t>COSE214, COSE221, COSE222, COSE341</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -4138,12 +4138,12 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>COSE214, COSE221, COSE342</t>
+          <t>COSE221, COSE222, COSE342</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -4153,13 +4153,13 @@
         <v>0.963</v>
       </c>
       <c r="E111" t="n">
-        <v>1.0352</v>
+        <v>1.0617</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>COSE211, COSE221, COSE341</t>
+          <t>COSE213, COSE221, COSE342</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -4180,12 +4180,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE222, COSE342</t>
+          <t>COSE214, COSE221, COSE342</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -4195,18 +4195,18 @@
         <v>0.963</v>
       </c>
       <c r="E113" t="n">
-        <v>1.0617</v>
+        <v>1.1502</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>COSE213, COSE221, COSE222, COSE341</t>
+          <t>COSE213, COSE221, COSE342</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -4216,13 +4216,13 @@
         <v>0.963</v>
       </c>
       <c r="E114" t="n">
-        <v>1.0617</v>
+        <v>1.1502</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>COSE213, COSE221, COSE342</t>
+          <t>COSE211, COSE213, COSE221, COSE222</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -4243,12 +4243,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE222, COSE342</t>
+          <t>COSE213, COSE221, COSE222, COSE341</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -4258,13 +4258,13 @@
         <v>0.963</v>
       </c>
       <c r="E116" t="n">
-        <v>1.1191</v>
+        <v>1.0617</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>COSE211, COSE222, COSE341, COSE342</t>
+          <t>COSE211, COSE213, COSE222, COSE342</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -4285,12 +4285,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>COSE211, COSE221, COSE341</t>
+          <t>COSE211, COSE214, COSE222, COSE342</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -4300,18 +4300,18 @@
         <v>0.963</v>
       </c>
       <c r="E118" t="n">
-        <v>1.1502</v>
+        <v>1.0352</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>COSE214, COSE221, COSE342</t>
+          <t>COSE221, COSE222, COSE342</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -4321,7 +4321,7 @@
         <v>0.963</v>
       </c>
       <c r="E119" t="n">
-        <v>1.1502</v>
+        <v>1.0352</v>
       </c>
     </row>
     <row r="120">
@@ -4332,7 +4332,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -4342,7 +4342,7 @@
         <v>0.963</v>
       </c>
       <c r="E120" t="n">
-        <v>1.0352</v>
+        <v>1.0617</v>
       </c>
     </row>
     <row r="121">
@@ -4369,12 +4369,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>COSE221, COSE222, COSE342</t>
+          <t>COSE213, COSE214, COSE221, COSE341</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -4384,18 +4384,18 @@
         <v>0.963</v>
       </c>
       <c r="E122" t="n">
-        <v>1.0617</v>
+        <v>1.1502</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE221, COSE222</t>
+          <t>COSE211, COSE221, COSE341</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -4405,18 +4405,18 @@
         <v>0.963</v>
       </c>
       <c r="E123" t="n">
-        <v>1.0617</v>
+        <v>1.1502</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>COSE211, COSE214, COSE221, COSE222</t>
+          <t>COSE211, COSE213, COSE222, COSE342</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -4426,18 +4426,18 @@
         <v>0.963</v>
       </c>
       <c r="E124" t="n">
-        <v>1.0352</v>
+        <v>1.1191</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>COSE213, COSE214, COSE221, COSE341</t>
+          <t>COSE211, COSE222, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -4447,18 +4447,18 @@
         <v>0.963</v>
       </c>
       <c r="E125" t="n">
-        <v>1.1502</v>
+        <v>1.0617</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE214, COSE221</t>
+          <t>COSE211, COSE222, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -4468,18 +4468,18 @@
         <v>0.963</v>
       </c>
       <c r="E126" t="n">
-        <v>1.1502</v>
+        <v>1.0352</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>COSE211, COSE222, COSE341, COSE342</t>
+          <t>COSE211, COSE213, COSE214, COSE221</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -4489,18 +4489,18 @@
         <v>0.963</v>
       </c>
       <c r="E127" t="n">
-        <v>1.0352</v>
+        <v>1.1502</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>COSE213, COSE221, COSE342</t>
+          <t>COSE211, COSE214, COSE221, COSE222</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -4510,13 +4510,13 @@
         <v>0.963</v>
       </c>
       <c r="E128" t="n">
-        <v>1.1502</v>
+        <v>1.0352</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>COSE221, COSE222, COSE342</t>
+          <t>COSE211, COSE221, COSE341</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -4563,7 +4563,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -4573,7 +4573,7 @@
         <v>0.9459</v>
       </c>
       <c r="E131" t="n">
-        <v>1.0169</v>
+        <v>1.043</v>
       </c>
     </row>
     <row r="132">
@@ -4605,7 +4605,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -4615,7 +4615,7 @@
         <v>0.9459</v>
       </c>
       <c r="E133" t="n">
-        <v>1.043</v>
+        <v>1.0169</v>
       </c>
     </row>
     <row r="134">
@@ -4626,7 +4626,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -4636,7 +4636,7 @@
         <v>0.9444</v>
       </c>
       <c r="E134" t="n">
-        <v>1.0413</v>
+        <v>1.0153</v>
       </c>
     </row>
     <row r="135">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -4678,7 +4678,7 @@
         <v>0.9444</v>
       </c>
       <c r="E136" t="n">
-        <v>1.0153</v>
+        <v>1.0413</v>
       </c>
     </row>
     <row r="137">
@@ -4726,12 +4726,12 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>COSE213, COSE214, COSE341</t>
+          <t>COSE222, COSE341</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE213, COSE214</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -4741,18 +4741,18 @@
         <v>0.9394</v>
       </c>
       <c r="E139" t="n">
-        <v>1.1221</v>
+        <v>1.063</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>COSE221</t>
+          <t>COSE213, COSE214, COSE341</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -4762,7 +4762,7 @@
         <v>0.9394</v>
       </c>
       <c r="E140" t="n">
-        <v>1.0098</v>
+        <v>1.1221</v>
       </c>
     </row>
     <row r="141">
@@ -4773,7 +4773,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -4783,18 +4783,18 @@
         <v>0.9394</v>
       </c>
       <c r="E141" t="n">
-        <v>1.0357</v>
+        <v>1.0098</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>COSE222, COSE341</t>
+          <t>COSE221</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>COSE213, COSE214</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -4804,7 +4804,7 @@
         <v>0.9394</v>
       </c>
       <c r="E142" t="n">
-        <v>1.063</v>
+        <v>1.0357</v>
       </c>
     </row>
     <row r="143">
@@ -4831,12 +4831,12 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>COSE211, COSE342</t>
+          <t>COSE211, COSE222</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -4846,18 +4846,18 @@
         <v>0.9375</v>
       </c>
       <c r="E144" t="n">
-        <v>1.0337</v>
+        <v>1.0895</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>COSE222, COSE342</t>
+          <t>COSE211, COSE341</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -4867,18 +4867,18 @@
         <v>0.9375</v>
       </c>
       <c r="E145" t="n">
-        <v>1.0895</v>
+        <v>1.1198</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>COSE211, COSE341</t>
+          <t>COSE211, COSE342</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>COSE213, COSE214</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -4888,18 +4888,18 @@
         <v>0.9375</v>
       </c>
       <c r="E146" t="n">
-        <v>1.0609</v>
+        <v>1.0337</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>COSE341, COSE342</t>
+          <t>COSE222, COSE342</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE213, COSE214</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -4909,18 +4909,18 @@
         <v>0.9375</v>
       </c>
       <c r="E147" t="n">
-        <v>1.1198</v>
+        <v>1.0609</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>COSE211, COSE341</t>
+          <t>COSE222, COSE342</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -4930,13 +4930,13 @@
         <v>0.9375</v>
       </c>
       <c r="E148" t="n">
-        <v>1.1198</v>
+        <v>1.0895</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>COSE211, COSE222</t>
+          <t>COSE211, COSE341</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4957,12 +4957,12 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>COSE211, COSE222</t>
+          <t>COSE211, COSE342</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -4972,13 +4972,13 @@
         <v>0.9375</v>
       </c>
       <c r="E150" t="n">
-        <v>1.0895</v>
+        <v>1.0078</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>COSE341, COSE342</t>
+          <t>COSE211, COSE222</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4999,12 +4999,12 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>COSE222, COSE342</t>
+          <t>COSE341, COSE342</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>COSE213, COSE214</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -5014,18 +5014,18 @@
         <v>0.9375</v>
       </c>
       <c r="E152" t="n">
-        <v>1.0609</v>
+        <v>1.1198</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>COSE211, COSE342</t>
+          <t>COSE341, COSE342</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE213, COSE214</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -5035,18 +5035,18 @@
         <v>0.9375</v>
       </c>
       <c r="E153" t="n">
-        <v>1.0078</v>
+        <v>1.0609</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE222</t>
+          <t>COSE215</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -5056,18 +5056,18 @@
         <v>0.9355</v>
       </c>
       <c r="E154" t="n">
-        <v>1.0872</v>
+        <v>1.0314</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE341</t>
+          <t>COSE214, COSE222, COSE342</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -5077,18 +5077,18 @@
         <v>0.9355</v>
       </c>
       <c r="E155" t="n">
-        <v>1.1174</v>
+        <v>1.0872</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>COSE213, COSE222, COSE342</t>
+          <t>COSE214, COSE221</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE213, COSE222</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -5098,7 +5098,7 @@
         <v>0.9355</v>
       </c>
       <c r="E156" t="n">
-        <v>1.0872</v>
+        <v>1.1493</v>
       </c>
     </row>
     <row r="157">
@@ -5125,7 +5125,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>COSE214, COSE341, COSE342</t>
+          <t>COSE213, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -5146,12 +5146,12 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>COSE213, COSE221</t>
+          <t>COSE211, COSE213, COSE222</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>COSE214, COSE222</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -5161,18 +5161,18 @@
         <v>0.9355</v>
       </c>
       <c r="E159" t="n">
-        <v>1.1493</v>
+        <v>1.0872</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>COSE215</t>
+          <t>COSE211, COSE214, COSE341</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>COSE213, COSE214</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -5182,18 +5182,18 @@
         <v>0.9355</v>
       </c>
       <c r="E160" t="n">
-        <v>1.0586</v>
+        <v>1.1174</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>COSE214, COSE222, COSE342</t>
+          <t>COSE215</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE213, COSE214</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -5203,18 +5203,18 @@
         <v>0.9355</v>
       </c>
       <c r="E161" t="n">
-        <v>1.0872</v>
+        <v>1.0586</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>COSE221, COSE222</t>
+          <t>COSE211, COSE214, COSE222</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>COSE213, COSE214</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -5224,18 +5224,18 @@
         <v>0.9355</v>
       </c>
       <c r="E162" t="n">
-        <v>1.0586</v>
+        <v>1.0872</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>COSE215</t>
+          <t>COSE213, COSE221</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE214, COSE222</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -5245,18 +5245,18 @@
         <v>0.9355</v>
       </c>
       <c r="E163" t="n">
-        <v>1.0314</v>
+        <v>1.1493</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>COSE214, COSE221</t>
+          <t>COSE211, COSE213, COSE341</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>COSE213, COSE222</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -5266,18 +5266,18 @@
         <v>0.9355</v>
       </c>
       <c r="E164" t="n">
-        <v>1.1493</v>
+        <v>1.1174</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>COSE211, COSE214, COSE341</t>
+          <t>COSE213, COSE222, COSE342</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -5287,18 +5287,18 @@
         <v>0.9355</v>
       </c>
       <c r="E165" t="n">
-        <v>1.1174</v>
+        <v>1.0872</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>COSE211, COSE214, COSE222</t>
+          <t>COSE221, COSE222</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE213, COSE214</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -5308,13 +5308,13 @@
         <v>0.9355</v>
       </c>
       <c r="E166" t="n">
-        <v>1.0872</v>
+        <v>1.0586</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>COSE213, COSE341, COSE342</t>
+          <t>COSE214, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -5335,12 +5335,12 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>COSE213, COSE215</t>
+          <t>COSE211, COSE221</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>COSE211, COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -5350,18 +5350,18 @@
         <v>0.9333</v>
       </c>
       <c r="E168" t="n">
-        <v>1.1467</v>
+        <v>1.0033</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>COSE211, COSE215</t>
+          <t>COSE371</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>COSE213, COSE214</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -5371,7 +5371,7 @@
         <v>0.9333</v>
       </c>
       <c r="E169" t="n">
-        <v>1.0561</v>
+        <v>1.0847</v>
       </c>
     </row>
     <row r="170">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>COSE342</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -5398,12 +5398,12 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>COSE211, COSE221</t>
+          <t>COSE371</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE213, COSE222</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -5413,18 +5413,18 @@
         <v>0.9333</v>
       </c>
       <c r="E171" t="n">
-        <v>1.0033</v>
+        <v>1.1467</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>COSE371</t>
+          <t>COSE213, COSE371</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>COSE213, COSE342</t>
+          <t>COSE342</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -5434,18 +5434,18 @@
         <v>0.9333</v>
       </c>
       <c r="E172" t="n">
-        <v>1.1804</v>
+        <v>1.1148</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>COSE371</t>
+          <t>COSE211, COSE221</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -5455,7 +5455,7 @@
         <v>0.9333</v>
       </c>
       <c r="E173" t="n">
-        <v>1.0847</v>
+        <v>1.1148</v>
       </c>
     </row>
     <row r="174">
@@ -5466,7 +5466,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE342</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -5482,12 +5482,12 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>COSE371</t>
+          <t>COSE211, COSE215</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>COSE342</t>
+          <t>COSE213, COSE214</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -5497,18 +5497,18 @@
         <v>0.9333</v>
       </c>
       <c r="E175" t="n">
-        <v>1.1148</v>
+        <v>1.0561</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>COSE213, COSE371</t>
+          <t>COSE213, COSE214, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -5518,18 +5518,18 @@
         <v>0.9333</v>
       </c>
       <c r="E176" t="n">
-        <v>1.0847</v>
+        <v>1.1148</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>COSE371</t>
+          <t>COSE213, COSE215</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>COSE213, COSE341</t>
+          <t>COSE211, COSE214</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -5545,12 +5545,12 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>COSE211, COSE221</t>
+          <t>COSE222, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE213, COSE214</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -5560,18 +5560,18 @@
         <v>0.9333</v>
       </c>
       <c r="E178" t="n">
-        <v>1.1148</v>
+        <v>1.0561</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>COSE211, COSE221</t>
+          <t>COSE213, COSE371</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -5581,18 +5581,18 @@
         <v>0.9333</v>
       </c>
       <c r="E179" t="n">
-        <v>1.0291</v>
+        <v>1.0847</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>COSE222, COSE341, COSE342</t>
+          <t>COSE371</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>COSE213, COSE214</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -5602,18 +5602,18 @@
         <v>0.9333</v>
       </c>
       <c r="E180" t="n">
-        <v>1.0561</v>
+        <v>1.1148</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>COSE213, COSE371</t>
+          <t>COSE371</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE213, COSE341</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -5623,18 +5623,18 @@
         <v>0.9333</v>
       </c>
       <c r="E181" t="n">
-        <v>1.1148</v>
+        <v>1.1467</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>COSE213, COSE214, COSE341, COSE342</t>
+          <t>COSE213, COSE214, COSE222, COSE342</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -5644,13 +5644,13 @@
         <v>0.9333</v>
       </c>
       <c r="E182" t="n">
-        <v>1.1148</v>
+        <v>1.0847</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>COSE211, COSE215</t>
+          <t>COSE211, COSE221</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -5671,7 +5671,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>COSE213, COSE214, COSE222, COSE342</t>
+          <t>COSE211, COSE214, COSE342</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -5692,12 +5692,12 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>COSE211, COSE214, COSE342</t>
+          <t>COSE211, COSE215</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -5707,13 +5707,13 @@
         <v>0.9333</v>
       </c>
       <c r="E185" t="n">
-        <v>1.0847</v>
+        <v>1.0291</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE342</t>
+          <t>COSE211, COSE213, COSE214, COSE222</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -5755,12 +5755,12 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE214, COSE222</t>
+          <t>COSE211, COSE213, COSE214, COSE341</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -5770,18 +5770,18 @@
         <v>0.9333</v>
       </c>
       <c r="E188" t="n">
-        <v>1.0847</v>
+        <v>1.1148</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE214, COSE341</t>
+          <t>COSE211, COSE213, COSE342</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -5791,7 +5791,7 @@
         <v>0.9333</v>
       </c>
       <c r="E189" t="n">
-        <v>1.1148</v>
+        <v>1.0847</v>
       </c>
     </row>
     <row r="190">
@@ -5802,7 +5802,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>COSE213, COSE222</t>
+          <t>COSE213, COSE342</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -5812,18 +5812,18 @@
         <v>0.9333</v>
       </c>
       <c r="E190" t="n">
-        <v>1.1467</v>
+        <v>1.1804</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>COSE214, COSE371</t>
+          <t>COSE221, COSE342</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>COSE342</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -5833,18 +5833,18 @@
         <v>0.931</v>
       </c>
       <c r="E191" t="n">
-        <v>1.1121</v>
+        <v>1.0265</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>COSE221, COSE342</t>
+          <t>COSE214, COSE371</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE213, COSE341</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -5854,18 +5854,18 @@
         <v>0.931</v>
       </c>
       <c r="E192" t="n">
-        <v>1.1121</v>
+        <v>1.1438</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>COSE221, COSE341</t>
+          <t>COSE211, COSE213, COSE214, COSE342</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>COSE213, COSE214</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -5875,18 +5875,18 @@
         <v>0.931</v>
       </c>
       <c r="E193" t="n">
-        <v>1.0535</v>
+        <v>1.082</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>COSE214, COSE371</t>
+          <t>COSE221, COSE342</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -5896,18 +5896,18 @@
         <v>0.931</v>
       </c>
       <c r="E194" t="n">
-        <v>1.1121</v>
+        <v>1.0009</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>COSE211, COSE341, COSE342</t>
+          <t>COSE213, COSE214, COSE371</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -5917,18 +5917,18 @@
         <v>0.931</v>
       </c>
       <c r="E195" t="n">
-        <v>1.1121</v>
+        <v>1.082</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>COSE213, COSE214, COSE371</t>
+          <t>COSE221, COSE341</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE214, COSE222</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -5938,18 +5938,18 @@
         <v>0.931</v>
       </c>
       <c r="E196" t="n">
-        <v>1.1121</v>
+        <v>1.1438</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>COSE221, COSE341</t>
+          <t>COSE214, COSE371</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>COSE213, COSE222</t>
+          <t>COSE342</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -5959,18 +5959,18 @@
         <v>0.931</v>
       </c>
       <c r="E197" t="n">
-        <v>1.1438</v>
+        <v>1.1121</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>COSE214, COSE371</t>
+          <t>COSE211, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>COSE213, COSE342</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -5980,18 +5980,18 @@
         <v>0.931</v>
       </c>
       <c r="E198" t="n">
-        <v>1.1775</v>
+        <v>1.1121</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>COSE214, COSE371</t>
+          <t>COSE213, COSE214, COSE371</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -6001,18 +6001,18 @@
         <v>0.931</v>
       </c>
       <c r="E199" t="n">
-        <v>1.082</v>
+        <v>1.1121</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>COSE214, COSE371</t>
+          <t>COSE221, COSE341</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>COSE213, COSE222</t>
+          <t>COSE213, COSE214</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -6022,18 +6022,18 @@
         <v>0.931</v>
       </c>
       <c r="E200" t="n">
-        <v>1.1438</v>
+        <v>1.0535</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>COSE213, COSE214, COSE371</t>
+          <t>COSE211, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE213, COSE214</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -6043,18 +6043,18 @@
         <v>0.931</v>
       </c>
       <c r="E201" t="n">
-        <v>1.082</v>
+        <v>1.0535</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>COSE221, COSE342</t>
+          <t>COSE214, COSE371</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>COSE213</t>
+          <t>COSE213, COSE342</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -6064,7 +6064,7 @@
         <v>0.931</v>
       </c>
       <c r="E202" t="n">
-        <v>1.0009</v>
+        <v>1.1775</v>
       </c>
     </row>
     <row r="203">
@@ -6075,7 +6075,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>COSE213, COSE341</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -6085,18 +6085,18 @@
         <v>0.931</v>
       </c>
       <c r="E203" t="n">
-        <v>1.1438</v>
+        <v>1.1121</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>COSE213, COSE214, COSE371</t>
+          <t>COSE221, COSE342</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>COSE342</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -6112,12 +6112,12 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE214, COSE342</t>
+          <t>COSE221, COSE341</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE213, COSE222</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -6127,18 +6127,18 @@
         <v>0.931</v>
       </c>
       <c r="E205" t="n">
-        <v>1.082</v>
+        <v>1.1438</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>COSE211, COSE341, COSE342</t>
+          <t>COSE214, COSE371</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>COSE213, COSE214</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -6148,7 +6148,7 @@
         <v>0.931</v>
       </c>
       <c r="E206" t="n">
-        <v>1.0535</v>
+        <v>1.082</v>
       </c>
     </row>
     <row r="207">
@@ -6159,7 +6159,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>COSE214, COSE222</t>
+          <t>COSE211</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -6169,18 +6169,18 @@
         <v>0.931</v>
       </c>
       <c r="E207" t="n">
-        <v>1.1438</v>
+        <v>1.082</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>COSE221, COSE342</t>
+          <t>COSE214, COSE371</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213, COSE222</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -6190,18 +6190,18 @@
         <v>0.931</v>
       </c>
       <c r="E208" t="n">
-        <v>1.0265</v>
+        <v>1.1438</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>COSE221, COSE341</t>
+          <t>COSE213, COSE214, COSE371</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>COSE211</t>
+          <t>COSE342</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -6211,18 +6211,18 @@
         <v>0.931</v>
       </c>
       <c r="E209" t="n">
-        <v>1.082</v>
+        <v>1.1121</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE221</t>
+          <t>COSE342, COSE371</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -6232,18 +6232,18 @@
         <v>0.9286</v>
       </c>
       <c r="E210" t="n">
-        <v>1.0792</v>
+        <v>1.1091</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE341, COSE342</t>
+          <t>COSE222, COSE371</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -6253,13 +6253,13 @@
         <v>0.9286</v>
       </c>
       <c r="E211" t="n">
-        <v>1.1091</v>
+        <v>1.0792</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>COSE221, COSE222, COSE341</t>
+          <t>COSE211, COSE221, COSE222</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -6280,12 +6280,12 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>COSE213, COSE221, COSE341</t>
+          <t>COSE211, COSE222, COSE342</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>COSE214, COSE222</t>
+          <t>COSE213, COSE214</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -6295,18 +6295,18 @@
         <v>0.9286</v>
       </c>
       <c r="E213" t="n">
-        <v>1.1408</v>
+        <v>1.0508</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>COSE341, COSE371</t>
+          <t>COSE222, COSE371</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE342</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -6322,12 +6322,12 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>COSE214, COSE221, COSE341</t>
+          <t>COSE211, COSE213, COSE221</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>COSE213, COSE222</t>
+          <t>COSE214, COSE222</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -6343,12 +6343,12 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE221</t>
+          <t>COSE211, COSE221, COSE222</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>COSE214, COSE222</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -6358,18 +6358,18 @@
         <v>0.9286</v>
       </c>
       <c r="E216" t="n">
-        <v>1.1408</v>
+        <v>1.0792</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>COSE211, COSE221, COSE222</t>
+          <t>COSE342, COSE371</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>COSE213, COSE214</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -6379,18 +6379,18 @@
         <v>0.9286</v>
       </c>
       <c r="E217" t="n">
-        <v>1.0508</v>
+        <v>1.0792</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>COSE211, COSE221, COSE222</t>
+          <t>COSE341, COSE371</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -6400,18 +6400,18 @@
         <v>0.9286</v>
       </c>
       <c r="E218" t="n">
-        <v>1.0792</v>
+        <v>1.1091</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>COSE211, COSE222, COSE342</t>
+          <t>COSE211, COSE213, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>COSE213, COSE341</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -6421,13 +6421,13 @@
         <v>0.9286</v>
       </c>
       <c r="E219" t="n">
-        <v>1.1408</v>
+        <v>1.1091</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>COSE222, COSE371</t>
+          <t>COSE341, COSE371</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -6448,12 +6448,12 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>COSE211, COSE214, COSE341, COSE342</t>
+          <t>COSE213, COSE221, COSE341</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE211</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -6463,7 +6463,7 @@
         <v>0.9286</v>
       </c>
       <c r="E221" t="n">
-        <v>1.1091</v>
+        <v>1.0792</v>
       </c>
     </row>
     <row r="222">
@@ -6474,7 +6474,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>COSE214, COSE341</t>
+          <t>COSE213, COSE341</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -6484,18 +6484,18 @@
         <v>0.9286</v>
       </c>
       <c r="E222" t="n">
-        <v>1.1744</v>
+        <v>1.1408</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>COSE211, COSE222, COSE342</t>
+          <t>COSE213, COSE341, COSE371</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>COSE213, COSE214</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -6505,18 +6505,18 @@
         <v>0.9286</v>
       </c>
       <c r="E223" t="n">
-        <v>1.0508</v>
+        <v>1.1091</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>COSE341, COSE371</t>
+          <t>COSE214, COSE221, COSE341</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>COSE213, COSE342</t>
+          <t>COSE213, COSE222</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -6526,18 +6526,18 @@
         <v>0.9286</v>
       </c>
       <c r="E224" t="n">
-        <v>1.1744</v>
+        <v>1.1408</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>COSE342, COSE371</t>
+          <t>COSE213, COSE221, COSE341</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>COSE213, COSE341</t>
+          <t>COSE214, COSE222</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -6553,12 +6553,12 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>COSE222, COSE371</t>
+          <t>COSE221, COSE222, COSE341</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE213, COSE214</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -6568,18 +6568,18 @@
         <v>0.9286</v>
       </c>
       <c r="E226" t="n">
-        <v>1.0792</v>
+        <v>1.0508</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>COSE213, COSE222, COSE371</t>
+          <t>COSE222, COSE371</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE213, COSE341</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -6589,13 +6589,13 @@
         <v>0.9286</v>
       </c>
       <c r="E227" t="n">
-        <v>1.0792</v>
+        <v>1.1408</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>COSE211, COSE214, COSE221</t>
+          <t>COSE341, COSE371</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6616,12 +6616,12 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>COSE214, COSE221, COSE341</t>
+          <t>COSE211, COSE214, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>COSE211</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -6631,18 +6631,18 @@
         <v>0.9286</v>
       </c>
       <c r="E229" t="n">
-        <v>1.0792</v>
+        <v>1.1091</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>COSE342, COSE371</t>
+          <t>COSE211, COSE222, COSE342</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE214, COSE341</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -6652,18 +6652,18 @@
         <v>0.9286</v>
       </c>
       <c r="E230" t="n">
-        <v>1.1091</v>
+        <v>1.1744</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>COSE222, COSE371</t>
+          <t>COSE213, COSE222, COSE371</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>COSE213, COSE342</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -6673,18 +6673,18 @@
         <v>0.9286</v>
       </c>
       <c r="E231" t="n">
-        <v>1.1744</v>
+        <v>1.0792</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>COSE341, COSE371</t>
+          <t>COSE222, COSE371</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>COSE342</t>
+          <t>COSE213, COSE342</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -6694,18 +6694,18 @@
         <v>0.9286</v>
       </c>
       <c r="E232" t="n">
-        <v>1.1091</v>
+        <v>1.1744</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>COSE342, COSE371</t>
+          <t>COSE213, COSE342, COSE371</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>COSE213, COSE222</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -6715,7 +6715,7 @@
         <v>0.9286</v>
       </c>
       <c r="E233" t="n">
-        <v>1.1408</v>
+        <v>1.1091</v>
       </c>
     </row>
     <row r="234">
@@ -6747,7 +6747,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE342</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -6763,12 +6763,12 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>COSE213, COSE342, COSE371</t>
+          <t>COSE211, COSE214, COSE221</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -6778,18 +6778,18 @@
         <v>0.9286</v>
       </c>
       <c r="E236" t="n">
-        <v>1.1091</v>
+        <v>1.0792</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>COSE342, COSE371</t>
+          <t>COSE214, COSE221, COSE341</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE211</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -6826,12 +6826,12 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>COSE213, COSE221, COSE341</t>
+          <t>COSE211, COSE214, COSE221</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>COSE211</t>
+          <t>COSE213, COSE222</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -6841,18 +6841,18 @@
         <v>0.9286</v>
       </c>
       <c r="E239" t="n">
-        <v>1.0792</v>
+        <v>1.1408</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>COSE222, COSE371</t>
+          <t>COSE341, COSE371</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>COSE213, COSE341</t>
+          <t>COSE213, COSE342</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -6862,18 +6862,18 @@
         <v>0.9286</v>
       </c>
       <c r="E240" t="n">
-        <v>1.1408</v>
+        <v>1.1744</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>COSE341, COSE371</t>
+          <t>COSE211, COSE213, COSE221</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>COSE213, COSE222</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -6883,18 +6883,18 @@
         <v>0.9286</v>
       </c>
       <c r="E241" t="n">
-        <v>1.1408</v>
+        <v>1.0792</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>COSE211, COSE214, COSE221</t>
+          <t>COSE342, COSE371</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE213, COSE341</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -6904,18 +6904,18 @@
         <v>0.9286</v>
       </c>
       <c r="E242" t="n">
-        <v>1.0792</v>
+        <v>1.1408</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>COSE213, COSE341, COSE371</t>
+          <t>COSE342, COSE371</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>COSE342</t>
+          <t>COSE213, COSE222</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -6925,7 +6925,7 @@
         <v>0.9286</v>
       </c>
       <c r="E243" t="n">
-        <v>1.1091</v>
+        <v>1.1408</v>
       </c>
     </row>
     <row r="244">
@@ -7120,12 +7120,12 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>COSE214, COSE341</t>
+          <t>COSE214, COSE342</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>COSE342</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -7135,18 +7135,18 @@
         <v>0.9118000000000001</v>
       </c>
       <c r="E253" t="n">
-        <v>1.0891</v>
+        <v>1.0596</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>COSE214, COSE342</t>
+          <t>COSE214, COSE341</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE342</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -7156,7 +7156,7 @@
         <v>0.9118000000000001</v>
       </c>
       <c r="E254" t="n">
-        <v>1.0596</v>
+        <v>1.0891</v>
       </c>
     </row>
     <row r="255">
@@ -7309,12 +7309,12 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>COSE213, COSE214, COSE341</t>
+          <t>COSE213, COSE214, COSE342</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>COSE342</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -7324,7 +7324,7 @@
         <v>0.9091</v>
       </c>
       <c r="E262" t="n">
-        <v>1.0859</v>
+        <v>1.0565</v>
       </c>
     </row>
     <row r="263">
@@ -7351,12 +7351,12 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>COSE213, COSE214, COSE342</t>
+          <t>COSE213, COSE214, COSE341</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE342</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -7366,7 +7366,7 @@
         <v>0.9091</v>
       </c>
       <c r="E264" t="n">
-        <v>1.0565</v>
+        <v>1.0859</v>
       </c>
     </row>
     <row r="265">
@@ -7498,12 +7498,12 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>COSE211, COSE341</t>
+          <t>COSE211, COSE222</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>COSE214, COSE222</t>
+          <t>COSE214, COSE341</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -7513,7 +7513,7 @@
         <v>0.9062</v>
       </c>
       <c r="E271" t="n">
-        <v>1.1134</v>
+        <v>1.1461</v>
       </c>
     </row>
     <row r="272">
@@ -7582,12 +7582,12 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>COSE211, COSE341</t>
+          <t>COSE341, COSE342</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>COSE342</t>
+          <t>COSE211</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -7597,18 +7597,18 @@
         <v>0.9062</v>
       </c>
       <c r="E275" t="n">
-        <v>1.0825</v>
+        <v>1.0532</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>COSE341, COSE342</t>
+          <t>COSE211, COSE342</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>COSE211</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -7624,12 +7624,12 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>COSE211, COSE342</t>
+          <t>COSE211, COSE341</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE342</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -7639,7 +7639,7 @@
         <v>0.9062</v>
       </c>
       <c r="E277" t="n">
-        <v>1.0532</v>
+        <v>1.0825</v>
       </c>
     </row>
     <row r="278">
@@ -7666,12 +7666,12 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>COSE211, COSE222</t>
+          <t>COSE211, COSE341</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>COSE214, COSE341</t>
+          <t>COSE214, COSE222</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -7681,7 +7681,7 @@
         <v>0.9062</v>
       </c>
       <c r="E279" t="n">
-        <v>1.1461</v>
+        <v>1.1134</v>
       </c>
     </row>
     <row r="280">
@@ -7876,12 +7876,12 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>COSE211, COSE214, COSE341</t>
+          <t>COSE214, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>COSE342</t>
+          <t>COSE211</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -7891,7 +7891,7 @@
         <v>0.9032</v>
       </c>
       <c r="E289" t="n">
-        <v>1.0789</v>
+        <v>1.0497</v>
       </c>
     </row>
     <row r="290">
@@ -8107,12 +8107,12 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>COSE214, COSE341, COSE342</t>
+          <t>COSE211, COSE214, COSE341</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>COSE211</t>
+          <t>COSE342</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -8122,7 +8122,7 @@
         <v>0.9032</v>
       </c>
       <c r="E300" t="n">
-        <v>1.0497</v>
+        <v>1.0789</v>
       </c>
     </row>
     <row r="301">
@@ -8233,12 +8233,12 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE341</t>
+          <t>COSE213, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>COSE342</t>
+          <t>COSE211</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -8248,18 +8248,18 @@
         <v>0.9032</v>
       </c>
       <c r="E306" t="n">
-        <v>1.0789</v>
+        <v>1.0497</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>COSE213, COSE341, COSE342</t>
+          <t>COSE211, COSE213, COSE341</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>COSE211</t>
+          <t>COSE342</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -8269,7 +8269,7 @@
         <v>0.9032</v>
       </c>
       <c r="E307" t="n">
-        <v>1.0497</v>
+        <v>1.0789</v>
       </c>
     </row>
     <row r="308">
@@ -8548,12 +8548,12 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>COSE214, COSE221, COSE222</t>
+          <t>COSE213, COSE214, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE211</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -8611,12 +8611,12 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>COSE211, COSE222, COSE341</t>
+          <t>COSE222, COSE341, COSE342</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>COSE342</t>
+          <t>COSE211</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -8626,18 +8626,18 @@
         <v>0.9</v>
       </c>
       <c r="E324" t="n">
-        <v>1.075</v>
+        <v>1.0459</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>COSE222, COSE341, COSE342</t>
+          <t>COSE211, COSE222, COSE341</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>COSE211</t>
+          <t>COSE342</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -8647,7 +8647,7 @@
         <v>0.9</v>
       </c>
       <c r="E325" t="n">
-        <v>1.0459</v>
+        <v>1.075</v>
       </c>
     </row>
     <row r="326">
@@ -8695,12 +8695,12 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>COSE211, COSE213, COSE214, COSE341</t>
+          <t>COSE211, COSE214, COSE342</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>COSE342</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -8716,12 +8716,12 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>COSE211, COSE214, COSE342</t>
+          <t>COSE214, COSE221, COSE222</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -8731,18 +8731,18 @@
         <v>0.9</v>
       </c>
       <c r="E329" t="n">
-        <v>1.075</v>
+        <v>1.0459</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>COSE213, COSE214, COSE341, COSE342</t>
+          <t>COSE211, COSE213, COSE214, COSE341</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>COSE211</t>
+          <t>COSE342</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -8752,7 +8752,7 @@
         <v>0.9</v>
       </c>
       <c r="E330" t="n">
-        <v>1.0459</v>
+        <v>1.075</v>
       </c>
     </row>
     <row r="331">

</xml_diff>